<commit_message>
feat(viceri-study): publish specification and test suite v1.3
</commit_message>
<xml_diff>
--- a/output/xlsx/AdministradorAdicionaAdministrador--GT-.xlsx
+++ b/output/xlsx/AdministradorAdicionaAdministrador--GT-.xlsx
@@ -116,7 +116,7 @@
     <t>Administrador: preenche os dados do Administrador, seleciona suas permissoes e clica no botao 'Registrar'</t>
   </si>
   <si>
-    <t>SYSTEM notifica que o Administrador foi adicionado com sucesso e exibe lista de Administradores</t>
+    <t>SYSTEM notifica que o Administrador foi adicionado com sucesso</t>
   </si>
   <si>
     <t xml:space="preserve">Postcondition: </t>
@@ -292,7 +292,7 @@
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="86.5546875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="79.20703125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="63.30078125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="17.578125" customWidth="true" bestFit="true"/>
   </cols>

</xml_diff>